<commit_message>
feat(auth): harden RBAC, add in-app password reset for admin, and update staging verification
</commit_message>
<xml_diff>
--- a/supabase/tests/artifacts/Bao_Cao_P7_4_Customer_Retention.xlsx
+++ b/supabase/tests/artifacts/Bao_Cao_P7_4_Customer_Retention.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>BÁO CÁO GIỮ CHÂN &amp; COHORT (P7.4)</t>
   </si>
@@ -97,16 +97,13 @@
     <t>0918111222</t>
   </si>
   <si>
-    <t>vip</t>
+    <t>gold</t>
   </si>
   <si>
     <t>Anh Hoàng Long</t>
   </si>
   <si>
     <t>0983333444</t>
-  </si>
-  <si>
-    <t>gold</t>
   </si>
 </sst>
 </file>
@@ -654,7 +651,7 @@
         <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E3">
         <v>0</v>

</xml_diff>